<commit_message>
adding plots and bulk upload
</commit_message>
<xml_diff>
--- a/static/template.xlsx
+++ b/static/template.xlsx
@@ -8,25 +8,37 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johan\Documents\python\st-fuel-log\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A60A23DF-EFCF-4E8F-8609-6D34F2B2B3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7829F5C4-99F6-4A7B-89CC-51296A914AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Input" sheetId="1" r:id="rId1"/>
-    <sheet name="metadata" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Fuel Entries" sheetId="1" r:id="rId1"/>
+    <sheet name="Vehicles" sheetId="3" r:id="rId2"/>
+    <sheet name="metadata" sheetId="2" state="hidden" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Vehicle</t>
   </si>
@@ -65,6 +77,27 @@
   </si>
   <si>
     <t>Odometer (km)</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Nickname</t>
+  </si>
+  <si>
+    <t>Registration Number</t>
+  </si>
+  <si>
+    <t>VIN Number</t>
+  </si>
+  <si>
+    <t>Model Description</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Registration Date</t>
   </si>
 </sst>
 </file>
@@ -88,7 +121,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -96,26 +129,177 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="5"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="5"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="5"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="5"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="5"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="5"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="5"/>
+        </left>
+        <top style="thin">
+          <color theme="5"/>
+        </top>
+        <bottom style="thin">
+          <color theme="5"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="5"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <border>
@@ -201,16 +385,16 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="datatreehouse" pivot="0" count="13" xr9:uid="{B9E32496-EFE3-417C-8A46-63EC059B2709}">
-      <tableStyleElement type="wholeTable" dxfId="10"/>
-      <tableStyleElement type="headerRow" dxfId="9"/>
-      <tableStyleElement type="totalRow" dxfId="8"/>
-      <tableStyleElement type="firstColumn" dxfId="7"/>
-      <tableStyleElement type="lastColumn" dxfId="6"/>
-      <tableStyleElement type="firstRowStripe" dxfId="5"/>
-      <tableStyleElement type="secondRowStripe" dxfId="4"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="3"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="2"/>
+    <tableStyle name="datatreehouse" pivot="0" count="9" xr9:uid="{B9E32496-EFE3-417C-8A46-63EC059B2709}">
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="secondRowStripe" dxfId="10"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="9"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="8"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -230,17 +414,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F6F931B-996C-400C-99CD-602EDE3D13C1}" name="Table1" displayName="Table1" ref="A1:H2" totalsRowShown="0">
-  <autoFilter ref="A1:H2" xr:uid="{7F6F931B-996C-400C-99CD-602EDE3D13C1}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{B8958D98-7B88-48FD-B94B-8BC24ED9A643}" name="Date (DD/MM/YYYY)" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F6F931B-996C-400C-99CD-602EDE3D13C1}" name="fuel_entries" displayName="fuel_entries" ref="A1:G2" totalsRowShown="0">
+  <autoFilter ref="A1:G2" xr:uid="{7F6F931B-996C-400C-99CD-602EDE3D13C1}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{B8958D98-7B88-48FD-B94B-8BC24ED9A643}" name="Date (DD/MM/YYYY)" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{3B27B583-0A63-4B86-BF55-82587619C500}" name="Vehicle"/>
     <tableColumn id="3" xr3:uid="{6C779F41-4748-4708-ADF5-250899A3686A}" name="Odometer (km)"/>
     <tableColumn id="4" xr3:uid="{8A4E126C-8164-4271-B41F-C37372AD64F0}" name="Trip Distance (km)"/>
     <tableColumn id="5" xr3:uid="{43966580-259B-4582-BEF6-048B307F7F7F}" name="Fuel Filled (Liters)"/>
-    <tableColumn id="6" xr3:uid="{40E47734-AF06-4A08-B583-3B3318DB2DD0}" name="Fuel Type"/>
     <tableColumn id="7" xr3:uid="{A0E319C5-5FBF-4CD7-A602-5ABB148BC771}" name="Price"/>
-    <tableColumn id="8" xr3:uid="{DC2E5365-E0FD-4A08-821E-E0AF83635C6B}" name="Location" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{DC2E5365-E0FD-4A08-821E-E0AF83635C6B}" name="Location" dataDxfId="6"/>
+  </tableColumns>
+  <tableStyleInfo name="datatreehouse" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CA3119E0-B46B-46A4-9FC6-704BD0EC37B8}" name="vehicles" displayName="vehicles" ref="A1:H2" insertRow="1" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:H2" xr:uid="{CA3119E0-B46B-46A4-9FC6-704BD0EC37B8}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{54FEED1A-7342-461A-AAE3-8F1082CFAE4A}" name="Id" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{BFC175C7-ED25-4AC0-BA78-B94BD1F80D22}" name="Nickname" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{0FA64E71-214F-4059-AFB7-FB83724614C7}" name="Fuel Type"/>
+    <tableColumn id="4" xr3:uid="{465C71BB-DEAB-42FD-9422-F0CB866477E7}" name="Registration Number"/>
+    <tableColumn id="5" xr3:uid="{CAEE8B77-7137-4B06-984E-FDFF5C8C6FC9}" name="VIN Number"/>
+    <tableColumn id="6" xr3:uid="{63D55BA8-DA60-4D8D-AE63-DA60E800A5E0}" name="Model Description"/>
+    <tableColumn id="7" xr3:uid="{FB008FCA-D740-4A4B-BF7D-78567FA14A18}" name="Color"/>
+    <tableColumn id="8" xr3:uid="{68243487-9EB9-4A5B-BED4-DAAFD05CABC8}" name="Registration Date"/>
   </tableColumns>
   <tableStyleInfo name="datatreehouse" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -512,19 +712,18 @@
   <sheetPr>
     <tabColor rgb="FFF36441"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
-    <col min="2" max="2" width="20.5546875" customWidth="1"/>
-    <col min="3" max="3" width="18.33203125" customWidth="1"/>
-    <col min="4" max="5" width="18.44140625" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" customWidth="1"/>
-    <col min="7" max="7" width="14.44140625" customWidth="1"/>
-    <col min="8" max="8" width="26.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="4" max="5" width="18.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="26.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -541,16 +740,13 @@
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
     </row>
   </sheetData>
@@ -558,50 +754,93 @@
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DF59EA1C-0DFC-4FC3-AD93-84C4385231BF}">
-          <x14:formula1>
-            <xm:f>metadata!$A$1:$A$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>F2</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D2BF63A-BF92-426B-8625-684F4775FA27}">
+  <sheetPr>
+    <tabColor rgb="FFF36441"/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="5"/>
+      <c r="B2" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F2EFDF7-0DC6-4B02-8CF0-0F9188646DCC}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
refactor: better bulk upload approach
</commit_message>
<xml_diff>
--- a/static/template.xlsx
+++ b/static/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johan\Documents\python\st-fuel-log\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A60A23DF-EFCF-4E8F-8609-6D34F2B2B3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89E74066-2AFF-49E7-8F9A-87C83B4610EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Input" sheetId="1" r:id="rId1"/>
@@ -26,18 +26,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
-  <si>
-    <t>Vehicle</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Trip Distance (km)</t>
   </si>
   <si>
     <t>Fuel Filled (Liters)</t>
-  </si>
-  <si>
-    <t>Fuel Type</t>
   </si>
   <si>
     <t>Price</t>
@@ -112,10 +106,10 @@
   </cellStyles>
   <dxfs count="11">
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border>
@@ -201,7 +195,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="datatreehouse" pivot="0" count="13" xr9:uid="{B9E32496-EFE3-417C-8A46-63EC059B2709}">
+    <tableStyle name="datatreehouse" pivot="0" count="9" xr9:uid="{B9E32496-EFE3-417C-8A46-63EC059B2709}">
       <tableStyleElement type="wholeTable" dxfId="10"/>
       <tableStyleElement type="headerRow" dxfId="9"/>
       <tableStyleElement type="totalRow" dxfId="8"/>
@@ -230,17 +224,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F6F931B-996C-400C-99CD-602EDE3D13C1}" name="Table1" displayName="Table1" ref="A1:H2" totalsRowShown="0">
-  <autoFilter ref="A1:H2" xr:uid="{7F6F931B-996C-400C-99CD-602EDE3D13C1}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{B8958D98-7B88-48FD-B94B-8BC24ED9A643}" name="Date (DD/MM/YYYY)" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{3B27B583-0A63-4B86-BF55-82587619C500}" name="Vehicle"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F6F931B-996C-400C-99CD-602EDE3D13C1}" name="Table1" displayName="Table1" ref="A1:F2" totalsRowShown="0">
+  <autoFilter ref="A1:F2" xr:uid="{7F6F931B-996C-400C-99CD-602EDE3D13C1}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{B8958D98-7B88-48FD-B94B-8BC24ED9A643}" name="Date (DD/MM/YYYY)" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{6C779F41-4748-4708-ADF5-250899A3686A}" name="Odometer (km)"/>
     <tableColumn id="4" xr3:uid="{8A4E126C-8164-4271-B41F-C37372AD64F0}" name="Trip Distance (km)"/>
     <tableColumn id="5" xr3:uid="{43966580-259B-4582-BEF6-048B307F7F7F}" name="Fuel Filled (Liters)"/>
-    <tableColumn id="6" xr3:uid="{40E47734-AF06-4A08-B583-3B3318DB2DD0}" name="Fuel Type"/>
     <tableColumn id="7" xr3:uid="{A0E319C5-5FBF-4CD7-A602-5ABB148BC771}" name="Price"/>
-    <tableColumn id="8" xr3:uid="{DC2E5365-E0FD-4A08-821E-E0AF83635C6B}" name="Location" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{DC2E5365-E0FD-4A08-821E-E0AF83635C6B}" name="Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="datatreehouse" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -512,27 +504,25 @@
   <sheetPr>
     <tabColor rgb="FFF36441"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.88671875" customWidth="1"/>
-    <col min="2" max="2" width="20.5546875" customWidth="1"/>
-    <col min="3" max="3" width="18.33203125" customWidth="1"/>
-    <col min="4" max="5" width="18.44140625" customWidth="1"/>
-    <col min="6" max="6" width="20.33203125" customWidth="1"/>
-    <col min="7" max="7" width="14.44140625" customWidth="1"/>
-    <col min="8" max="8" width="26.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="3" max="4" width="18.44140625" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" customWidth="1"/>
+    <col min="6" max="6" width="26.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>12</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -540,17 +530,11 @@
       <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
     </row>
   </sheetData>
@@ -558,18 +542,6 @@
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DF59EA1C-0DFC-4FC3-AD93-84C4385231BF}">
-          <x14:formula1>
-            <xm:f>metadata!$A$1:$A$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>F2</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -583,27 +555,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>